<commit_message>
Making it faster according to gpt
</commit_message>
<xml_diff>
--- a/case_studies/base_case_5_dd/2025/technologies.xlsx
+++ b/case_studies/base_case_5_dd/2025/technologies.xlsx
@@ -1064,7 +1064,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>62.79</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0</v>
@@ -1073,19 +1073,19 @@
         <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0</v>
+        <v>11.11</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
+        <v>24.41</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>46.83</v>
+        <v>95.48999999999999</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
+        <v>42.99</v>
       </c>
       <c r="L6" s="3" t="n">
         <v>0</v>
@@ -1130,7 +1130,7 @@
         <v>0</v>
       </c>
       <c r="Z6" s="3" t="n">
-        <v>0</v>
+        <v>59.12</v>
       </c>
       <c r="AA6" s="3" t="n">
         <v>0</v>

</xml_diff>